<commit_message>
solved bugs and Leave excel upload
</commit_message>
<xml_diff>
--- a/web/src/main/webapp/StorageYard/Other/UserDoc/LeaveExcelUpload/LeaveExcelUpload.xlsx
+++ b/web/src/main/webapp/StorageYard/Other/UserDoc/LeaveExcelUpload/LeaveExcelUpload.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
@@ -16,28 +16,34 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Employee No</t>
   </si>
   <si>
-    <t xml:space="preserve"> Casual Leave </t>
-  </si>
-  <si>
     <t>Sick Leave</t>
   </si>
   <si>
     <t>Privilege Leave</t>
   </si>
   <si>
-    <t>Paternity Leave</t>
+    <t>National Holiday</t>
+  </si>
+  <si>
+    <t>Lieu Day Leave</t>
+  </si>
+  <si>
+    <t>Casual Leave</t>
+  </si>
+  <si>
+    <t>656644</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -74,17 +80,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -163,6 +175,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -197,6 +210,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -372,32 +386,56 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.28515625" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
     <col min="4" max="4" width="20.28515625" customWidth="1"/>
     <col min="5" max="5" width="20.85546875" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -407,18 +445,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Changes in Salary Report (Arrears and Deductions).
</commit_message>
<xml_diff>
--- a/web/src/main/webapp/StorageYard/Other/UserDoc/LeaveExcelUpload/LeaveExcelUpload.xlsx
+++ b/web/src/main/webapp/StorageYard/Other/UserDoc/LeaveExcelUpload/LeaveExcelUpload.xlsx
@@ -30,13 +30,13 @@
     <t>National Holiday</t>
   </si>
   <si>
-    <t>Lieu Day Leave</t>
-  </si>
-  <si>
     <t>Casual Leave</t>
   </si>
   <si>
     <t>656644</t>
+  </si>
+  <si>
+    <t>Leave Without Pay</t>
   </si>
 </sst>
 </file>
@@ -403,7 +403,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -412,7 +412,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -420,7 +420,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2">
         <v>10</v>

</xml_diff>